<commit_message>
cambios en api gemini
</commit_message>
<xml_diff>
--- a/data/pedidos.xlsx
+++ b/data/pedidos.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -516,6 +516,186 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>1789751287-2kq2xt</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>18/09/2026 17:08</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>web-a47s8f</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>1.0x Hielo bolsa 2kg</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>confirmado</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>1789752240-vkolz9</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>18/09/2026 17:24</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>web-q1apks</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>1.0x Coca-Cola 500ml</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>1800</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>confirmado</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>1789760768-k9j0x5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>18/09/2026 19:46</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>web-dqr230</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>1.0x Hielo bolsa 2kg</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>confirmado</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1790101513-hb25gf</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>22/09/2026 18:25</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>web-9hukzo</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>6.0x Coca-Cola 500ml</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>10800</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>confirmado</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1790101632-6zznpi</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>22/09/2026 18:27</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>web-co17tb</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2.0x Coca-Cola 500ml</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>3600</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>confirmado</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1790107232-095gtb</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>22/09/2026 20:00</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>web-h5ogij</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>1.0x Paquete de galletitas Oreo</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>2100</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>confirmado</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>